<commit_message>
Seeding project bulk data
</commit_message>
<xml_diff>
--- a/public/assets/excel/employee_office_infos.xlsx
+++ b/public/assets/excel/employee_office_infos.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="29231"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="24326"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Asus\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo LOQ\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8BF0143-1D90-4987-A79D-BCD4D15B26F9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A02F23FC-C32F-4DB1-89D6-5BC42CB4C84E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
@@ -109,9 +109,6 @@
     <t xml:space="preserve">10th </t>
   </si>
   <si>
-    <t>Tofsil A</t>
-  </si>
-  <si>
     <t>Company 1</t>
   </si>
   <si>
@@ -242,6 +239,9 @@
   </si>
   <si>
     <t>Maxime eaque molliti</t>
+  </si>
+  <si>
+    <t>Act A</t>
   </si>
 </sst>
 </file>
@@ -590,172 +590,172 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:AM3"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="13.7265625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.6328125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.36328125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.1796875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="21.1796875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="28.08984375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18.6328125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="23.453125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="23.1796875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="10.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="21.81640625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="20.7265625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="20.453125" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="24.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.6640625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="9.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="21.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="28.109375" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="18.6640625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="23.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="23.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="10.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="20.77734375" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="20.44140625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="24.109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="20" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="23.81640625" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="21" max="21" width="20.36328125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="23.77734375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="21" max="21" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="18" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="19.36328125" bestFit="1" customWidth="1"/>
-    <col min="24" max="24" width="15.26953125" bestFit="1" customWidth="1"/>
-    <col min="25" max="25" width="16.6328125" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="17.36328125" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="28" max="28" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="19.33203125" bestFit="1" customWidth="1"/>
+    <col min="24" max="24" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="25" max="25" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="28" max="28" width="19.21875" bestFit="1" customWidth="1"/>
     <col min="29" max="29" width="18" bestFit="1" customWidth="1"/>
-    <col min="30" max="30" width="32.90625" bestFit="1" customWidth="1"/>
-    <col min="31" max="31" width="19.90625" bestFit="1" customWidth="1"/>
-    <col min="32" max="32" width="10.36328125" bestFit="1" customWidth="1"/>
-    <col min="33" max="33" width="21.7265625" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="35" max="35" width="16.81640625" bestFit="1" customWidth="1"/>
-    <col min="36" max="36" width="11.90625" bestFit="1" customWidth="1"/>
-    <col min="37" max="37" width="27.36328125" bestFit="1" customWidth="1"/>
-    <col min="38" max="38" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="39" max="39" width="15.36328125" bestFit="1" customWidth="1"/>
-    <col min="40" max="40" width="17.81640625" bestFit="1" customWidth="1"/>
-    <col min="41" max="41" width="10.453125" bestFit="1" customWidth="1"/>
-    <col min="43" max="43" width="1.7265625" bestFit="1" customWidth="1"/>
+    <col min="30" max="30" width="32.88671875" bestFit="1" customWidth="1"/>
+    <col min="31" max="31" width="19.88671875" bestFit="1" customWidth="1"/>
+    <col min="32" max="32" width="10.33203125" bestFit="1" customWidth="1"/>
+    <col min="33" max="33" width="21.77734375" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="35" max="35" width="16.77734375" bestFit="1" customWidth="1"/>
+    <col min="36" max="36" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="37" max="37" width="27.33203125" bestFit="1" customWidth="1"/>
+    <col min="38" max="38" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="39" max="39" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="40" max="40" width="17.77734375" bestFit="1" customWidth="1"/>
+    <col min="41" max="41" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="43" max="43" width="1.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
       <c r="B1" t="s">
+        <v>35</v>
+      </c>
+      <c r="C1" t="s">
         <v>36</v>
-      </c>
-      <c r="C1" t="s">
-        <v>37</v>
       </c>
       <c r="D1" t="s">
         <v>1</v>
       </c>
       <c r="E1" t="s">
+        <v>37</v>
+      </c>
+      <c r="F1" t="s">
         <v>38</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>39</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>40</v>
       </c>
-      <c r="H1" t="s">
+      <c r="I1" t="s">
         <v>41</v>
       </c>
-      <c r="I1" t="s">
+      <c r="J1" t="s">
         <v>42</v>
       </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>43</v>
       </c>
-      <c r="K1" t="s">
+      <c r="L1" t="s">
         <v>44</v>
       </c>
-      <c r="L1" t="s">
+      <c r="M1" t="s">
         <v>45</v>
       </c>
-      <c r="M1" t="s">
+      <c r="N1" t="s">
         <v>46</v>
       </c>
-      <c r="N1" t="s">
+      <c r="O1" t="s">
         <v>47</v>
       </c>
-      <c r="O1" t="s">
+      <c r="P1" t="s">
         <v>48</v>
       </c>
-      <c r="P1" t="s">
+      <c r="Q1" t="s">
         <v>49</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="R1" t="s">
         <v>50</v>
       </c>
-      <c r="R1" t="s">
+      <c r="S1" t="s">
         <v>51</v>
       </c>
-      <c r="S1" t="s">
+      <c r="T1" t="s">
         <v>52</v>
       </c>
-      <c r="T1" t="s">
+      <c r="U1" t="s">
         <v>53</v>
       </c>
-      <c r="U1" t="s">
+      <c r="V1" t="s">
         <v>54</v>
       </c>
-      <c r="V1" t="s">
+      <c r="W1" t="s">
         <v>55</v>
       </c>
-      <c r="W1" t="s">
+      <c r="X1" t="s">
         <v>56</v>
       </c>
-      <c r="X1" t="s">
+      <c r="Y1" t="s">
         <v>57</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Z1" t="s">
         <v>58</v>
       </c>
-      <c r="Z1" t="s">
+      <c r="AA1" t="s">
         <v>59</v>
       </c>
-      <c r="AA1" t="s">
+      <c r="AB1" t="s">
         <v>60</v>
       </c>
-      <c r="AB1" t="s">
+      <c r="AC1" s="1" t="s">
         <v>61</v>
       </c>
-      <c r="AC1" s="1" t="s">
+      <c r="AD1" s="1" t="s">
         <v>62</v>
       </c>
-      <c r="AD1" s="1" t="s">
+      <c r="AE1" s="1" t="s">
         <v>63</v>
       </c>
-      <c r="AE1" s="1" t="s">
+      <c r="AF1" s="1" t="s">
         <v>64</v>
       </c>
-      <c r="AF1" s="1" t="s">
+      <c r="AG1" s="1" t="s">
         <v>65</v>
       </c>
-      <c r="AG1" s="1" t="s">
+      <c r="AH1" s="1" t="s">
         <v>66</v>
       </c>
-      <c r="AH1" s="1" t="s">
+      <c r="AI1" s="1" t="s">
         <v>67</v>
       </c>
-      <c r="AI1" s="1" t="s">
+      <c r="AJ1" s="1" t="s">
         <v>68</v>
       </c>
-      <c r="AJ1" s="1" t="s">
+      <c r="AK1" s="1" t="s">
         <v>69</v>
       </c>
-      <c r="AK1" s="1" t="s">
+      <c r="AL1" s="1" t="s">
         <v>70</v>
       </c>
-      <c r="AL1" s="1" t="s">
+      <c r="AM1" s="1" t="s">
         <v>71</v>
       </c>
-      <c r="AM1" s="1" t="s">
-        <v>72</v>
-      </c>
     </row>
-    <row r="2" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A2">
         <v>3422</v>
       </c>
@@ -769,49 +769,49 @@
         <v>983</v>
       </c>
       <c r="E2" t="s">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="F2" t="s">
         <v>3</v>
       </c>
       <c r="G2" t="s">
+        <v>29</v>
+      </c>
+      <c r="H2" t="s">
         <v>30</v>
       </c>
-      <c r="H2" t="s">
+      <c r="I2" t="s">
         <v>31</v>
       </c>
-      <c r="I2" t="s">
+      <c r="J2" t="s">
         <v>32</v>
       </c>
-      <c r="J2" t="s">
+      <c r="K2" t="s">
         <v>33</v>
       </c>
-      <c r="K2" t="s">
+      <c r="L2" t="s">
         <v>34</v>
-      </c>
-      <c r="L2" t="s">
-        <v>35</v>
       </c>
       <c r="M2" t="s">
         <v>4</v>
       </c>
       <c r="N2" t="s">
+        <v>29</v>
+      </c>
+      <c r="O2" t="s">
         <v>30</v>
       </c>
-      <c r="O2" t="s">
+      <c r="P2" t="s">
         <v>31</v>
       </c>
-      <c r="P2" t="s">
+      <c r="Q2" t="s">
         <v>32</v>
       </c>
-      <c r="Q2" t="s">
+      <c r="R2" t="s">
         <v>33</v>
       </c>
-      <c r="R2" t="s">
+      <c r="S2" t="s">
         <v>34</v>
-      </c>
-      <c r="S2" t="s">
-        <v>35</v>
       </c>
       <c r="T2" t="s">
         <v>5</v>
@@ -874,9 +874,9 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:39" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:39" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B3" t="s">
         <v>15</v>
@@ -888,49 +888,49 @@
         <v>303</v>
       </c>
       <c r="E3" t="s">
-        <v>29</v>
+        <v>73</v>
       </c>
       <c r="F3" t="s">
         <v>16</v>
       </c>
       <c r="G3" t="s">
+        <v>29</v>
+      </c>
+      <c r="H3" t="s">
         <v>30</v>
       </c>
-      <c r="H3" t="s">
+      <c r="I3" t="s">
         <v>31</v>
       </c>
-      <c r="I3" t="s">
+      <c r="J3" t="s">
         <v>32</v>
       </c>
-      <c r="J3" t="s">
+      <c r="K3" t="s">
         <v>33</v>
       </c>
-      <c r="K3" t="s">
+      <c r="L3" t="s">
         <v>34</v>
-      </c>
-      <c r="L3" t="s">
-        <v>35</v>
       </c>
       <c r="M3" t="s">
         <v>17</v>
       </c>
       <c r="N3" t="s">
+        <v>29</v>
+      </c>
+      <c r="O3" t="s">
         <v>30</v>
       </c>
-      <c r="O3" t="s">
+      <c r="P3" t="s">
         <v>31</v>
       </c>
-      <c r="P3" t="s">
+      <c r="Q3" t="s">
         <v>32</v>
       </c>
-      <c r="Q3" t="s">
+      <c r="R3" t="s">
         <v>33</v>
       </c>
-      <c r="R3" t="s">
+      <c r="S3" t="s">
         <v>34</v>
-      </c>
-      <c r="S3" t="s">
-        <v>35</v>
       </c>
       <c r="T3" t="s">
         <v>5</v>

</xml_diff>